<commit_message>
CI Reports [2026-06-25 20:55]: All — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report/Daily Reports/BugReport_25-Jun-2026.xlsx
+++ b/Test Execution Report/Daily Reports/BugReport_25-Jun-2026.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Bug Report" sheetId="1" r:id="rId1"/>
+    <sheet name="Daily Bug Report" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -398,371 +399,728 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:R6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Bug ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Title</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Module / Feature</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Linked TC ID</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Severity</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Priority</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Environment</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Steps to Reproduce</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Expected Result</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Actual Result</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Reported Date</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Reporter</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Screenshot / Evidence</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Bug Exists in Tracker</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Tracker Bug ID</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Tracker Status</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Remarks</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>BUG-DASHBOARD-MODULE-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>TC-DASH-002 | All 4 stat cards visible with values</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="D2" t="str">
+        <v>TC-DASH-002</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F2" t="str">
+        <v>P3</v>
+      </c>
+      <c r="G2" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="H2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="K2" t="str">
+        <v>New</v>
+      </c>
+      <c r="L2" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="M2" t="str">
+        <v>QA Automation</v>
+      </c>
+      <c r="N2" t="str">
+        <v>reports/screenshots/TC-DASH-002-failure.png</v>
+      </c>
+      <c r="O2" t="str">
+        <v>No</v>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v>New — not yet in tracker</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>BUG-DASHBOARD-MODULE-002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>TC-DASH-004 | ANALYTICS tab shows analytics content</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="D3" t="str">
+        <v>TC-DASH-004</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F3" t="str">
+        <v>P3</v>
+      </c>
+      <c r="G3" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="H3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="K3" t="str">
+        <v>New</v>
+      </c>
+      <c r="L3" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="M3" t="str">
+        <v>QA Automation</v>
+      </c>
+      <c r="N3" t="str">
+        <v>reports/screenshots/TC-DASH-004-failure.png</v>
+      </c>
+      <c r="O3" t="str">
+        <v>No</v>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v>New — not yet in tracker</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>BUG-DASHBOARD-MODULE-003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>TC-DASH-005 | Switch back to OVERVIEW from ANALYTICS</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="D4" t="str">
+        <v>TC-DASH-005</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F4" t="str">
+        <v>P3</v>
+      </c>
+      <c r="G4" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="H4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="K4" t="str">
+        <v>New</v>
+      </c>
+      <c r="L4" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="M4" t="str">
+        <v>QA Automation</v>
+      </c>
+      <c r="N4" t="str">
+        <v>reports/screenshots/TC-DASH-005-failure.png</v>
+      </c>
+      <c r="O4" t="str">
+        <v>No</v>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v>New — not yet in tracker</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>BUG-DASHBOARD-MODULE-004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>TC-DASH-007 | Reset button clears date filter</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="D5" t="str">
+        <v>TC-DASH-007</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F5" t="str">
+        <v>P3</v>
+      </c>
+      <c r="G5" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="H5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mlocator_x001b_[39m_x001b_[2m)._x001b_[22mtoBeVisible_x001b_[2m(_x001b_[22m_x001b_[2m)_x001b_[22m failed  Locator:  locator('button:has-text("Reset")').first() Expected: visible Received: hidden Timeout:  5000ms  Ca</v>
+      </c>
+      <c r="K5" t="str">
+        <v>New</v>
+      </c>
+      <c r="L5" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="M5" t="str">
+        <v>QA Automation</v>
+      </c>
+      <c r="N5" t="str">
+        <v>reports/screenshots/TC-DASH-007-failure.png</v>
+      </c>
+      <c r="O5" t="str">
+        <v>No</v>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v>New — not yet in tracker</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>BUG-DASHBOARD-MODULE-005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>TC-DASH-011 | All sidebar navigation links present</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="D6" t="str">
+        <v>TC-DASH-011</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F6" t="str">
+        <v>P3</v>
+      </c>
+      <c r="G6" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="H6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mlocator_x001b_[39m_x001b_[2m)._x001b_[22mtoBeVisible_x001b_[2m(_x001b_[22m_x001b_[2m)_x001b_[22m failed  Locator:  locator('a[href="/Ticket/Index"]').first() Expected: visible Received: hidden Timeout:  5000ms  Cal</v>
+      </c>
+      <c r="K6" t="str">
+        <v>New</v>
+      </c>
+      <c r="L6" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="M6" t="str">
+        <v>QA Automation</v>
+      </c>
+      <c r="N6" t="str">
+        <v>reports/screenshots/TC-DASH-011-failure.png</v>
+      </c>
+      <c r="O6" t="str">
+        <v>No</v>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v>New — not yet in tracker</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:R6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:R6"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="50.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
     <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="40.83203125" customWidth="1"/>
-    <col min="8" max="8" width="45.83203125" customWidth="1"/>
-    <col min="9" max="9" width="35.83203125" customWidth="1"/>
-    <col min="10" max="10" width="45.83203125" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" customWidth="1"/>
-    <col min="12" max="12" width="14.83203125" customWidth="1"/>
-    <col min="13" max="13" width="16.83203125" customWidth="1"/>
-    <col min="14" max="14" width="45.83203125" customWidth="1"/>
-    <col min="15" max="15" width="22.83203125" customWidth="1"/>
-    <col min="16" max="16" width="16.83203125" customWidth="1"/>
-    <col min="17" max="17" width="16.83203125" customWidth="1"/>
-    <col min="18" max="18" width="35.83203125" customWidth="1"/>
+    <col min="4" max="4" width="44.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="44.83203125" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="36.83203125" customWidth="1"/>
+    <col min="13" max="13" width="10.83203125" customWidth="1"/>
+    <col min="14" max="14" width="10.83203125" customWidth="1"/>
+    <col min="15" max="15" width="40.83203125" customWidth="1"/>
+    <col min="16" max="16" width="32.83203125" customWidth="1"/>
+    <col min="17" max="17" width="44.83203125" customWidth="1"/>
+    <col min="18" max="18" width="36.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Bug ID</v>
+        <v>Date</v>
       </c>
       <c r="B1" t="str">
-        <v>Title</v>
+        <v>Module</v>
       </c>
       <c r="C1" t="str">
-        <v>Module / Feature</v>
+        <v>TC ID</v>
       </c>
       <c r="D1" t="str">
-        <v>Linked TC ID</v>
+        <v>Test Case Name</v>
       </c>
       <c r="E1" t="str">
-        <v>Severity</v>
+        <v>Test Type</v>
       </c>
       <c r="F1" t="str">
         <v>Priority</v>
       </c>
       <c r="G1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Bug ID</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Bug Title</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Severity</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Bug Priority</v>
+      </c>
+      <c r="L1" t="str">
         <v>Environment</v>
       </c>
-      <c r="H1" t="str">
+      <c r="M1" t="str">
+        <v>Browser</v>
+      </c>
+      <c r="N1" t="str">
+        <v>OS</v>
+      </c>
+      <c r="O1" t="str">
         <v>Steps to Reproduce</v>
       </c>
-      <c r="I1" t="str">
+      <c r="P1" t="str">
         <v>Expected Result</v>
       </c>
-      <c r="J1" t="str">
+      <c r="Q1" t="str">
         <v>Actual Result</v>
       </c>
-      <c r="K1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Reported Date</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Reporter</v>
-      </c>
-      <c r="N1" t="str">
-        <v>Screenshot / Evidence</v>
-      </c>
-      <c r="O1" t="str">
-        <v>Bug Exists in Tracker</v>
-      </c>
-      <c r="P1" t="str">
-        <v>Tracker Bug ID</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>Tracker Status</v>
-      </c>
       <c r="R1" t="str">
-        <v>Remarks</v>
+        <v>Source Report</v>
       </c>
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="C2" t="str">
+        <v>TC-DASH-002</v>
+      </c>
+      <c r="D2" t="str">
+        <v>TC-DASH-002 | All 4 stat cards visible with values</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G2" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H2" t="str">
         <v>BUG-DASHBOARD-MODULE-001</v>
       </c>
-      <c r="B2" t="str">
-        <v>TC-DASH-002 | All 4 stat cards visible with values</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Dashboard Module</v>
-      </c>
-      <c r="D2" t="str">
-        <v>TC-DASH-002</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Low</v>
-      </c>
-      <c r="F2" t="str">
+      <c r="I2" t="str">
+        <v>[FAIL] TC-DASH-002 | All 4 stat cards visible with values</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K2" t="str">
         <v>P3</v>
       </c>
-      <c r="G2" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
-      </c>
-      <c r="H2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate
-2. Execute test
+      <c r="L2" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to feature page
+2. Execute test steps
 3. Observe failure</v>
       </c>
-      <c r="I2" t="str">
-        <v>Test should pass</v>
-      </c>
-      <c r="J2" t="str">
+      <c r="P2" t="str">
+        <v>Test should pass successfully</v>
+      </c>
+      <c r="Q2" t="str">
         <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
       </c>
-      <c r="K2" t="str">
-        <v>New</v>
-      </c>
-      <c r="L2" t="str">
-        <v>25 Jun 2026</v>
-      </c>
-      <c r="M2" t="str">
-        <v>QA Automation</v>
-      </c>
-      <c r="N2" t="str">
-        <v>reports/screenshots/TC-DASH-002-failure.png</v>
-      </c>
-      <c r="O2" t="str">
-        <v>No</v>
-      </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
-      <c r="Q2" t="str">
-        <v/>
-      </c>
       <c r="R2" t="str">
-        <v>New — not yet in tracker</v>
+        <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="C3" t="str">
+        <v>TC-DASH-004</v>
+      </c>
+      <c r="D3" t="str">
+        <v>TC-DASH-004 | ANALYTICS tab shows analytics content</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G3" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H3" t="str">
         <v>BUG-DASHBOARD-MODULE-002</v>
       </c>
-      <c r="B3" t="str">
-        <v>TC-DASH-004 | ANALYTICS tab shows analytics content</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Dashboard Module</v>
-      </c>
-      <c r="D3" t="str">
-        <v>TC-DASH-004</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Low</v>
-      </c>
-      <c r="F3" t="str">
+      <c r="I3" t="str">
+        <v>[FAIL] TC-DASH-004 | ANALYTICS tab shows analytics content</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K3" t="str">
         <v>P3</v>
       </c>
-      <c r="G3" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
-      </c>
-      <c r="H3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate
-2. Execute test
+      <c r="L3" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to feature page
+2. Execute test steps
 3. Observe failure</v>
       </c>
-      <c r="I3" t="str">
-        <v>Test should pass</v>
-      </c>
-      <c r="J3" t="str">
+      <c r="P3" t="str">
+        <v>Test should pass successfully</v>
+      </c>
+      <c r="Q3" t="str">
         <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
       </c>
-      <c r="K3" t="str">
-        <v>New</v>
-      </c>
-      <c r="L3" t="str">
-        <v>25 Jun 2026</v>
-      </c>
-      <c r="M3" t="str">
-        <v>QA Automation</v>
-      </c>
-      <c r="N3" t="str">
-        <v>reports/screenshots/TC-DASH-004-failure.png</v>
-      </c>
-      <c r="O3" t="str">
-        <v>No</v>
-      </c>
-      <c r="P3" t="str">
-        <v/>
-      </c>
-      <c r="Q3" t="str">
-        <v/>
-      </c>
       <c r="R3" t="str">
-        <v>New — not yet in tracker</v>
+        <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
       <c r="A4" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="C4" t="str">
+        <v>TC-DASH-005</v>
+      </c>
+      <c r="D4" t="str">
+        <v>TC-DASH-005 | Switch back to OVERVIEW from ANALYTICS</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G4" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H4" t="str">
         <v>BUG-DASHBOARD-MODULE-003</v>
       </c>
-      <c r="B4" t="str">
-        <v>TC-DASH-005 | Switch back to OVERVIEW from ANALYTICS</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Dashboard Module</v>
-      </c>
-      <c r="D4" t="str">
-        <v>TC-DASH-005</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Low</v>
-      </c>
-      <c r="F4" t="str">
+      <c r="I4" t="str">
+        <v>[FAIL] TC-DASH-005 | Switch back to OVERVIEW from ANALYTICS</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K4" t="str">
         <v>P3</v>
       </c>
-      <c r="G4" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
-      </c>
-      <c r="H4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate
-2. Execute test
+      <c r="L4" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to feature page
+2. Execute test steps
 3. Observe failure</v>
       </c>
-      <c r="I4" t="str">
-        <v>Test should pass</v>
-      </c>
-      <c r="J4" t="str">
+      <c r="P4" t="str">
+        <v>Test should pass successfully</v>
+      </c>
+      <c r="Q4" t="str">
         <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
       </c>
-      <c r="K4" t="str">
-        <v>New</v>
-      </c>
-      <c r="L4" t="str">
-        <v>25 Jun 2026</v>
-      </c>
-      <c r="M4" t="str">
-        <v>QA Automation</v>
-      </c>
-      <c r="N4" t="str">
-        <v>reports/screenshots/TC-DASH-005-failure.png</v>
-      </c>
-      <c r="O4" t="str">
-        <v>No</v>
-      </c>
-      <c r="P4" t="str">
-        <v/>
-      </c>
-      <c r="Q4" t="str">
-        <v/>
-      </c>
       <c r="R4" t="str">
-        <v>New — not yet in tracker</v>
+        <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
       </c>
     </row>
     <row r="5" xml:space="preserve">
       <c r="A5" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="C5" t="str">
+        <v>TC-DASH-007</v>
+      </c>
+      <c r="D5" t="str">
+        <v>TC-DASH-007 | Reset button clears date filter</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G5" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H5" t="str">
         <v>BUG-DASHBOARD-MODULE-004</v>
       </c>
-      <c r="B5" t="str">
-        <v>TC-DASH-007 | Reset button clears date filter</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Dashboard Module</v>
-      </c>
-      <c r="D5" t="str">
-        <v>TC-DASH-007</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Low</v>
-      </c>
-      <c r="F5" t="str">
+      <c r="I5" t="str">
+        <v>[FAIL] TC-DASH-007 | Reset button clears date filter</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K5" t="str">
         <v>P3</v>
       </c>
-      <c r="G5" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
-      </c>
-      <c r="H5" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate
-2. Execute test
+      <c r="L5" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to feature page
+2. Execute test steps
 3. Observe failure</v>
       </c>
-      <c r="I5" t="str">
-        <v>Test should pass</v>
-      </c>
-      <c r="J5" t="str">
+      <c r="P5" t="str">
+        <v>Test should pass successfully</v>
+      </c>
+      <c r="Q5" t="str">
         <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mlocator_x001b_[39m_x001b_[2m)._x001b_[22mtoBeVisible_x001b_[2m(_x001b_[22m_x001b_[2m)_x001b_[22m failed  Locator:  locator('button:has-text("Reset")').first() Expected: visible Received: hidden Timeout:  5000ms  Ca</v>
       </c>
-      <c r="K5" t="str">
-        <v>New</v>
-      </c>
-      <c r="L5" t="str">
-        <v>25 Jun 2026</v>
-      </c>
-      <c r="M5" t="str">
-        <v>QA Automation</v>
-      </c>
-      <c r="N5" t="str">
-        <v>reports/screenshots/TC-DASH-007-failure.png</v>
-      </c>
-      <c r="O5" t="str">
-        <v>No</v>
-      </c>
-      <c r="P5" t="str">
-        <v/>
-      </c>
-      <c r="Q5" t="str">
-        <v/>
-      </c>
       <c r="R5" t="str">
-        <v>New — not yet in tracker</v>
+        <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
       </c>
     </row>
     <row r="6" xml:space="preserve">
       <c r="A6" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="C6" t="str">
+        <v>TC-DASH-011</v>
+      </c>
+      <c r="D6" t="str">
+        <v>TC-DASH-011 | All sidebar navigation links present</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G6" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H6" t="str">
         <v>BUG-DASHBOARD-MODULE-005</v>
       </c>
-      <c r="B6" t="str">
-        <v>TC-DASH-011 | All sidebar navigation links present</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Dashboard Module</v>
-      </c>
-      <c r="D6" t="str">
-        <v>TC-DASH-011</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Low</v>
-      </c>
-      <c r="F6" t="str">
+      <c r="I6" t="str">
+        <v>[FAIL] TC-DASH-011 | All sidebar navigation links present</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K6" t="str">
         <v>P3</v>
       </c>
-      <c r="G6" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
-      </c>
-      <c r="H6" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate
-2. Execute test
+      <c r="L6" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to feature page
+2. Execute test steps
 3. Observe failure</v>
       </c>
-      <c r="I6" t="str">
-        <v>Test should pass</v>
-      </c>
-      <c r="J6" t="str">
+      <c r="P6" t="str">
+        <v>Test should pass successfully</v>
+      </c>
+      <c r="Q6" t="str">
         <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mlocator_x001b_[39m_x001b_[2m)._x001b_[22mtoBeVisible_x001b_[2m(_x001b_[22m_x001b_[2m)_x001b_[22m failed  Locator:  locator('a[href="/Ticket/Index"]').first() Expected: visible Received: hidden Timeout:  5000ms  Cal</v>
       </c>
-      <c r="K6" t="str">
-        <v>New</v>
-      </c>
-      <c r="L6" t="str">
-        <v>25 Jun 2026</v>
-      </c>
-      <c r="M6" t="str">
-        <v>QA Automation</v>
-      </c>
-      <c r="N6" t="str">
-        <v>reports/screenshots/TC-DASH-011-failure.png</v>
-      </c>
-      <c r="O6" t="str">
-        <v>No</v>
-      </c>
-      <c r="P6" t="str">
-        <v/>
-      </c>
-      <c r="Q6" t="str">
-        <v/>
-      </c>
       <c r="R6" t="str">
-        <v>New — not yet in tracker</v>
+        <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CI Reports [2026-06-25 21:25]: All — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report/Daily Reports/BugReport_25-Jun-2026.xlsx
+++ b/Test Execution Report/Daily Reports/BugReport_25-Jun-2026.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:R6"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -475,9 +475,299 @@
         <v>Source Report</v>
       </c>
     </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="C2" t="str">
+        <v>TC-DASH-002</v>
+      </c>
+      <c r="D2" t="str">
+        <v>TC-DASH-002 | All 4 stat cards visible with values</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G2" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H2" t="str">
+        <v>BUG-DASHBOARD-MODULE-001</v>
+      </c>
+      <c r="I2" t="str">
+        <v>[FAIL] TC-DASH-002 | All 4 stat cards visible with values</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K2" t="str">
+        <v>P3</v>
+      </c>
+      <c r="L2" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to feature page
+2. Execute test steps
+3. Observe failure</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Test should pass successfully</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="C3" t="str">
+        <v>TC-DASH-004</v>
+      </c>
+      <c r="D3" t="str">
+        <v>TC-DASH-004 | ANALYTICS tab shows analytics content</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G3" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H3" t="str">
+        <v>BUG-DASHBOARD-MODULE-002</v>
+      </c>
+      <c r="I3" t="str">
+        <v>[FAIL] TC-DASH-004 | ANALYTICS tab shows analytics content</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K3" t="str">
+        <v>P3</v>
+      </c>
+      <c r="L3" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to feature page
+2. Execute test steps
+3. Observe failure</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Test should pass successfully</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="R3" t="str">
+        <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="C4" t="str">
+        <v>TC-DASH-005</v>
+      </c>
+      <c r="D4" t="str">
+        <v>TC-DASH-005 | Switch back to OVERVIEW from ANALYTICS</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G4" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H4" t="str">
+        <v>BUG-DASHBOARD-MODULE-003</v>
+      </c>
+      <c r="I4" t="str">
+        <v>[FAIL] TC-DASH-005 | Switch back to OVERVIEW from ANALYTICS</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K4" t="str">
+        <v>P3</v>
+      </c>
+      <c r="L4" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to feature page
+2. Execute test steps
+3. Observe failure</v>
+      </c>
+      <c r="P4" t="str">
+        <v>Test should pass successfully</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="R4" t="str">
+        <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="C5" t="str">
+        <v>TC-DASH-011</v>
+      </c>
+      <c r="D5" t="str">
+        <v>TC-DASH-011 | All sidebar navigation links present</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G5" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H5" t="str">
+        <v>BUG-DASHBOARD-MODULE-004</v>
+      </c>
+      <c r="I5" t="str">
+        <v>[FAIL] TC-DASH-011 | All sidebar navigation links present</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K5" t="str">
+        <v>P3</v>
+      </c>
+      <c r="L5" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to feature page
+2. Execute test steps
+3. Observe failure</v>
+      </c>
+      <c r="P5" t="str">
+        <v>Test should pass successfully</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mlocator_x001b_[39m_x001b_[2m)._x001b_[22mtoBeVisible_x001b_[2m(_x001b_[22m_x001b_[2m)_x001b_[22m failed  Locator:  locator('a[href="/Ticket/Index"]').first() Expected: visible Received: hidden Timeout:  5000ms  Cal</v>
+      </c>
+      <c r="R5" t="str">
+        <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="C6" t="str">
+        <v>TC-DASH-012</v>
+      </c>
+      <c r="D6" t="str">
+        <v>TC-DASH-012 | Action Queue badge shows ticket count</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G6" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H6" t="str">
+        <v>BUG-DASHBOARD-MODULE-005</v>
+      </c>
+      <c r="I6" t="str">
+        <v>[FAIL] TC-DASH-012 | Action Queue badge shows ticket count</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K6" t="str">
+        <v>P3</v>
+      </c>
+      <c r="L6" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to feature page
+2. Execute test steps
+3. Observe failure</v>
+      </c>
+      <c r="P6" t="str">
+        <v>Test should pass successfully</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="R6" t="str">
+        <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>